<commit_message>
feat: implement Twitter data extraction module with configuration and CI/CD build support
</commit_message>
<xml_diff>
--- a/X月新番完结评分.xlsx
+++ b/X月新番完结评分.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\python\mzzbscore\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{795253B4-5CA9-43AB-A102-825E36B3A3D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73D88F9C-F4C4-4D29-9C9B-B1C7EEB8B33B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="3195" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,9 +37,6 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
-  <si>
-    <t>2025年XX月新番X期评分（数据截止日期XXXX年XX月XX日）</t>
-  </si>
   <si>
     <t>原名</t>
   </si>
@@ -159,12 +156,16 @@
     <t>排名差</t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
+  <si>
+    <t>2026年XX月新番X期评分（数据截止日期XXXX年XX月XX日）</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="176" formatCode="0.000_);[Red]\(0.000\)"/>
     <numFmt numFmtId="177" formatCode="0.00_);[Red]\(0.00\)"/>
     <numFmt numFmtId="178" formatCode="0.0_);[Red]\(0.0\)"/>
@@ -172,6 +173,7 @@
     <numFmt numFmtId="180" formatCode="0_ "/>
     <numFmt numFmtId="181" formatCode="0.000_ "/>
     <numFmt numFmtId="182" formatCode="0.0_ "/>
+    <numFmt numFmtId="183" formatCode="0_);[Red]\(0\)"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -413,7 +415,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -719,10 +721,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -738,6 +736,35 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="179" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="183" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="3" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="12" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="5" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1037,30 +1064,32 @@
     <col min="14" max="14" width="14" style="7" customWidth="1"/>
     <col min="15" max="17" width="14.109375" style="8" customWidth="1"/>
     <col min="18" max="25" width="17" style="9" customWidth="1"/>
-    <col min="26" max="35" width="17.88671875" style="9" customWidth="1"/>
+    <col min="26" max="27" width="17.88671875" style="9" customWidth="1"/>
+    <col min="28" max="28" width="17.88671875" style="118" customWidth="1"/>
+    <col min="29" max="35" width="17.88671875" style="9" customWidth="1"/>
     <col min="36" max="36" width="43.109375" style="1" customWidth="1"/>
     <col min="37" max="37" width="49.88671875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:928" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="103" t="s">
-        <v>0</v>
+      <c r="A1" s="110" t="s">
+        <v>35</v>
       </c>
-      <c r="B1" s="104"/>
-      <c r="C1" s="104"/>
-      <c r="D1" s="104"/>
-      <c r="E1" s="104"/>
-      <c r="F1" s="104"/>
-      <c r="G1" s="104"/>
-      <c r="H1" s="104"/>
-      <c r="I1" s="104"/>
-      <c r="J1" s="104"/>
-      <c r="K1" s="104"/>
-      <c r="L1" s="104"/>
-      <c r="M1" s="104"/>
-      <c r="N1" s="104"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="111"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="111"/>
       <c r="R1" s="7">
-        <v>20250714</v>
+        <v>20260410</v>
       </c>
       <c r="S1" s="7"/>
       <c r="T1" s="7"/>
@@ -1071,7 +1100,7 @@
       <c r="Y1" s="7"/>
       <c r="Z1" s="7"/>
       <c r="AA1" s="7"/>
-      <c r="AB1" s="7"/>
+      <c r="AB1" s="112"/>
       <c r="AC1" s="7"/>
       <c r="AD1" s="7"/>
       <c r="AE1" s="7"/>
@@ -1082,109 +1111,109 @@
     </row>
     <row r="2" spans="1:928" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="103" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="105" t="s">
+      <c r="C2" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="60" t="s">
+      <c r="D2" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="60" t="s">
+      <c r="E2" s="104" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="106" t="s">
+      <c r="F2" s="59" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="59" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="105" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="59" t="s">
-        <v>22</v>
+      <c r="I2" s="60" t="s">
+        <v>6</v>
       </c>
-      <c r="G2" s="59" t="s">
+      <c r="J2" s="104" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="107" t="s">
-        <v>6</v>
+      <c r="L2" s="59" t="s">
+        <v>24</v>
       </c>
-      <c r="I2" s="60" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" s="106" t="s">
+      <c r="M2" s="105" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="59" t="s">
-        <v>24</v>
+      <c r="N2" s="60" t="s">
+        <v>9</v>
       </c>
-      <c r="L2" s="59" t="s">
+      <c r="O2" s="104" t="s">
+        <v>10</v>
+      </c>
+      <c r="P2" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="M2" s="107" t="s">
-        <v>9</v>
+      <c r="Q2" s="59" t="s">
+        <v>26</v>
       </c>
-      <c r="N2" s="60" t="s">
-        <v>10</v>
-      </c>
-      <c r="O2" s="106" t="s">
+      <c r="R2" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="59" t="s">
-        <v>26</v>
+      <c r="S2" s="60" t="s">
+        <v>12</v>
       </c>
-      <c r="Q2" s="59" t="s">
+      <c r="T2" s="104" t="s">
+        <v>13</v>
+      </c>
+      <c r="U2" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="R2" s="61" t="s">
-        <v>12</v>
+      <c r="V2" s="59" t="s">
+        <v>28</v>
       </c>
-      <c r="S2" s="60" t="s">
-        <v>13</v>
+      <c r="W2" s="59" t="s">
+        <v>32</v>
       </c>
-      <c r="T2" s="106" t="s">
+      <c r="X2" s="59" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y2" s="60" t="s">
+        <v>30</v>
+      </c>
+      <c r="Z2" s="60" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA2" s="60" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB2" s="113" t="s">
+        <v>34</v>
+      </c>
+      <c r="AC2" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="U2" s="59" t="s">
-        <v>28</v>
-      </c>
-      <c r="V2" s="59" t="s">
-        <v>29</v>
-      </c>
-      <c r="W2" s="59" t="s">
-        <v>33</v>
-      </c>
-      <c r="X2" s="59" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y2" s="60" t="s">
-        <v>31</v>
-      </c>
-      <c r="Z2" s="60" t="s">
-        <v>30</v>
-      </c>
-      <c r="AA2" s="60" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB2" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC2" s="60" t="s">
+      <c r="AD2" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="AD2" s="60" t="s">
+      <c r="AE2" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="AE2" s="60" t="s">
+      <c r="AF2" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="AF2" s="60" t="s">
+      <c r="AG2" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="AG2" s="60" t="s">
+      <c r="AH2" s="106" t="s">
         <v>19</v>
       </c>
-      <c r="AH2" s="108" t="s">
+      <c r="AI2" s="107" t="s">
         <v>20</v>
-      </c>
-      <c r="AI2" s="109" t="s">
-        <v>21</v>
       </c>
       <c r="AJ2" s="12"/>
       <c r="AK2" s="12"/>
@@ -2086,22 +2115,34 @@
       <c r="D3" s="16"/>
       <c r="E3" s="17"/>
       <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
+      <c r="G3" s="108">
+        <f>C3-F3</f>
+        <v>0</v>
+      </c>
       <c r="H3" s="18"/>
       <c r="I3" s="19"/>
       <c r="J3" s="20"/>
       <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
+      <c r="L3" s="31">
+        <f>H3-K3</f>
+        <v>0</v>
+      </c>
       <c r="M3" s="21"/>
       <c r="N3" s="22"/>
       <c r="O3" s="23"/>
       <c r="P3" s="23"/>
-      <c r="Q3" s="23"/>
+      <c r="Q3" s="109">
+        <f>M3-P3</f>
+        <v>0</v>
+      </c>
       <c r="R3" s="24"/>
       <c r="S3" s="24"/>
       <c r="T3" s="24"/>
       <c r="U3" s="24"/>
-      <c r="V3" s="24"/>
+      <c r="V3" s="24">
+        <f>S3-U3</f>
+        <v>0</v>
+      </c>
       <c r="W3" s="62">
         <f>C3*0.5+H3*0.2+M3*0.1+R3*0.2</f>
         <v>0</v>
@@ -2109,8 +2150,14 @@
       <c r="X3" s="62"/>
       <c r="Y3" s="62"/>
       <c r="Z3" s="62"/>
-      <c r="AA3" s="62"/>
-      <c r="AB3" s="62"/>
+      <c r="AA3" s="62">
+        <f>W3-Y3</f>
+        <v>0</v>
+      </c>
+      <c r="AB3" s="114">
+        <f>X3-Z3</f>
+        <v>0</v>
+      </c>
       <c r="AC3" s="72"/>
       <c r="AD3" s="72"/>
       <c r="AE3" s="82"/>
@@ -2147,7 +2194,7 @@
       <c r="Y4" s="63"/>
       <c r="Z4" s="63"/>
       <c r="AA4" s="63"/>
-      <c r="AB4" s="63"/>
+      <c r="AB4" s="114"/>
       <c r="AC4" s="73"/>
       <c r="AD4" s="73"/>
       <c r="AE4" s="83"/>
@@ -2186,7 +2233,7 @@
       <c r="Y5" s="63"/>
       <c r="Z5" s="63"/>
       <c r="AA5" s="63"/>
-      <c r="AB5" s="63"/>
+      <c r="AB5" s="114"/>
       <c r="AC5" s="73"/>
       <c r="AD5" s="73"/>
       <c r="AE5" s="83"/>
@@ -2223,7 +2270,7 @@
       <c r="Y6" s="63"/>
       <c r="Z6" s="63"/>
       <c r="AA6" s="63"/>
-      <c r="AB6" s="63"/>
+      <c r="AB6" s="114"/>
       <c r="AC6" s="73"/>
       <c r="AD6" s="73"/>
       <c r="AE6" s="83"/>
@@ -2260,7 +2307,7 @@
       <c r="Y7" s="63"/>
       <c r="Z7" s="63"/>
       <c r="AA7" s="63"/>
-      <c r="AB7" s="63"/>
+      <c r="AB7" s="114"/>
       <c r="AC7" s="73"/>
       <c r="AD7" s="73"/>
       <c r="AE7" s="83"/>
@@ -3189,7 +3236,7 @@
       <c r="Y8" s="63"/>
       <c r="Z8" s="63"/>
       <c r="AA8" s="63"/>
-      <c r="AB8" s="63"/>
+      <c r="AB8" s="114"/>
       <c r="AC8" s="73"/>
       <c r="AD8" s="73"/>
       <c r="AE8" s="83"/>
@@ -3226,7 +3273,7 @@
       <c r="Y9" s="63"/>
       <c r="Z9" s="63"/>
       <c r="AA9" s="63"/>
-      <c r="AB9" s="63"/>
+      <c r="AB9" s="114"/>
       <c r="AC9" s="73"/>
       <c r="AD9" s="73"/>
       <c r="AE9" s="83"/>
@@ -4156,7 +4203,7 @@
       <c r="Y10" s="63"/>
       <c r="Z10" s="63"/>
       <c r="AA10" s="63"/>
-      <c r="AB10" s="63"/>
+      <c r="AB10" s="114"/>
       <c r="AC10" s="73"/>
       <c r="AD10" s="73"/>
       <c r="AE10" s="83"/>
@@ -5085,7 +5132,7 @@
       <c r="Y11" s="63"/>
       <c r="Z11" s="63"/>
       <c r="AA11" s="63"/>
-      <c r="AB11" s="63"/>
+      <c r="AB11" s="114"/>
       <c r="AC11" s="73"/>
       <c r="AD11" s="73"/>
       <c r="AE11" s="83"/>
@@ -6015,7 +6062,7 @@
       <c r="Y12" s="63"/>
       <c r="Z12" s="63"/>
       <c r="AA12" s="63"/>
-      <c r="AB12" s="63"/>
+      <c r="AB12" s="114"/>
       <c r="AC12" s="73"/>
       <c r="AD12" s="73"/>
       <c r="AE12" s="83"/>
@@ -6944,7 +6991,7 @@
       <c r="Y13" s="63"/>
       <c r="Z13" s="63"/>
       <c r="AA13" s="63"/>
-      <c r="AB13" s="63"/>
+      <c r="AB13" s="114"/>
       <c r="AC13" s="73"/>
       <c r="AD13" s="73"/>
       <c r="AE13" s="83"/>
@@ -6981,7 +7028,7 @@
       <c r="Y14" s="63"/>
       <c r="Z14" s="63"/>
       <c r="AA14" s="63"/>
-      <c r="AB14" s="63"/>
+      <c r="AB14" s="114"/>
       <c r="AC14" s="73"/>
       <c r="AD14" s="73"/>
       <c r="AE14" s="83"/>
@@ -7018,7 +7065,7 @@
       <c r="Y15" s="63"/>
       <c r="Z15" s="63"/>
       <c r="AA15" s="63"/>
-      <c r="AB15" s="63"/>
+      <c r="AB15" s="114"/>
       <c r="AC15" s="73"/>
       <c r="AD15" s="73"/>
       <c r="AE15" s="83"/>
@@ -7055,7 +7102,7 @@
       <c r="Y16" s="63"/>
       <c r="Z16" s="63"/>
       <c r="AA16" s="63"/>
-      <c r="AB16" s="63"/>
+      <c r="AB16" s="114"/>
       <c r="AC16" s="73"/>
       <c r="AD16" s="73"/>
       <c r="AE16" s="83"/>
@@ -7984,7 +8031,7 @@
       <c r="Y17" s="63"/>
       <c r="Z17" s="63"/>
       <c r="AA17" s="63"/>
-      <c r="AB17" s="63"/>
+      <c r="AB17" s="114"/>
       <c r="AC17" s="73"/>
       <c r="AD17" s="73"/>
       <c r="AE17" s="83"/>
@@ -8021,7 +8068,7 @@
       <c r="Y18" s="63"/>
       <c r="Z18" s="63"/>
       <c r="AA18" s="63"/>
-      <c r="AB18" s="63"/>
+      <c r="AB18" s="114"/>
       <c r="AC18" s="73"/>
       <c r="AD18" s="73"/>
       <c r="AE18" s="83"/>
@@ -8950,7 +8997,7 @@
       <c r="Y19" s="63"/>
       <c r="Z19" s="63"/>
       <c r="AA19" s="63"/>
-      <c r="AB19" s="63"/>
+      <c r="AB19" s="114"/>
       <c r="AC19" s="73"/>
       <c r="AD19" s="73"/>
       <c r="AE19" s="83"/>
@@ -8987,7 +9034,7 @@
       <c r="Y20" s="63"/>
       <c r="Z20" s="63"/>
       <c r="AA20" s="63"/>
-      <c r="AB20" s="63"/>
+      <c r="AB20" s="114"/>
       <c r="AC20" s="73"/>
       <c r="AD20" s="73"/>
       <c r="AE20" s="83"/>
@@ -9916,7 +9963,7 @@
       <c r="Y21" s="63"/>
       <c r="Z21" s="63"/>
       <c r="AA21" s="63"/>
-      <c r="AB21" s="63"/>
+      <c r="AB21" s="114"/>
       <c r="AC21" s="73"/>
       <c r="AD21" s="73"/>
       <c r="AE21" s="83"/>
@@ -9953,7 +10000,7 @@
       <c r="Y22" s="63"/>
       <c r="Z22" s="63"/>
       <c r="AA22" s="63"/>
-      <c r="AB22" s="63"/>
+      <c r="AB22" s="114"/>
       <c r="AC22" s="73"/>
       <c r="AD22" s="73"/>
       <c r="AE22" s="83"/>
@@ -10882,7 +10929,7 @@
       <c r="Y23" s="63"/>
       <c r="Z23" s="63"/>
       <c r="AA23" s="63"/>
-      <c r="AB23" s="63"/>
+      <c r="AB23" s="114"/>
       <c r="AC23" s="73"/>
       <c r="AD23" s="73"/>
       <c r="AE23" s="83"/>
@@ -11811,7 +11858,7 @@
       <c r="Y24" s="63"/>
       <c r="Z24" s="63"/>
       <c r="AA24" s="63"/>
-      <c r="AB24" s="63"/>
+      <c r="AB24" s="114"/>
       <c r="AC24" s="73"/>
       <c r="AD24" s="73"/>
       <c r="AE24" s="83"/>
@@ -11848,7 +11895,7 @@
       <c r="Y25" s="63"/>
       <c r="Z25" s="63"/>
       <c r="AA25" s="63"/>
-      <c r="AB25" s="63"/>
+      <c r="AB25" s="114"/>
       <c r="AC25" s="73"/>
       <c r="AD25" s="73"/>
       <c r="AE25" s="83"/>
@@ -12777,7 +12824,7 @@
       <c r="Y26" s="63"/>
       <c r="Z26" s="63"/>
       <c r="AA26" s="63"/>
-      <c r="AB26" s="63"/>
+      <c r="AB26" s="114"/>
       <c r="AC26" s="73"/>
       <c r="AD26" s="73"/>
       <c r="AE26" s="83"/>
@@ -12814,7 +12861,7 @@
       <c r="Y27" s="63"/>
       <c r="Z27" s="63"/>
       <c r="AA27" s="63"/>
-      <c r="AB27" s="63"/>
+      <c r="AB27" s="114"/>
       <c r="AC27" s="73"/>
       <c r="AD27" s="73"/>
       <c r="AE27" s="83"/>
@@ -13743,7 +13790,7 @@
       <c r="Y28" s="63"/>
       <c r="Z28" s="63"/>
       <c r="AA28" s="63"/>
-      <c r="AB28" s="63"/>
+      <c r="AB28" s="114"/>
       <c r="AC28" s="73"/>
       <c r="AD28" s="73"/>
       <c r="AE28" s="83"/>
@@ -14672,7 +14719,7 @@
       <c r="Y29" s="63"/>
       <c r="Z29" s="63"/>
       <c r="AA29" s="63"/>
-      <c r="AB29" s="63"/>
+      <c r="AB29" s="114"/>
       <c r="AC29" s="73"/>
       <c r="AD29" s="73"/>
       <c r="AE29" s="83"/>
@@ -15601,7 +15648,7 @@
       <c r="Y30" s="63"/>
       <c r="Z30" s="63"/>
       <c r="AA30" s="63"/>
-      <c r="AB30" s="63"/>
+      <c r="AB30" s="114"/>
       <c r="AC30" s="73"/>
       <c r="AD30" s="73"/>
       <c r="AE30" s="83"/>
@@ -16530,7 +16577,7 @@
       <c r="Y31" s="63"/>
       <c r="Z31" s="63"/>
       <c r="AA31" s="63"/>
-      <c r="AB31" s="63"/>
+      <c r="AB31" s="114"/>
       <c r="AC31" s="73"/>
       <c r="AD31" s="73"/>
       <c r="AE31" s="83"/>
@@ -17459,7 +17506,7 @@
       <c r="Y32" s="63"/>
       <c r="Z32" s="63"/>
       <c r="AA32" s="63"/>
-      <c r="AB32" s="63"/>
+      <c r="AB32" s="114"/>
       <c r="AC32" s="73"/>
       <c r="AD32" s="73"/>
       <c r="AE32" s="83"/>
@@ -18388,7 +18435,7 @@
       <c r="Y33" s="63"/>
       <c r="Z33" s="63"/>
       <c r="AA33" s="63"/>
-      <c r="AB33" s="63"/>
+      <c r="AB33" s="114"/>
       <c r="AC33" s="73"/>
       <c r="AD33" s="73"/>
       <c r="AE33" s="83"/>
@@ -18425,7 +18472,7 @@
       <c r="Y34" s="63"/>
       <c r="Z34" s="63"/>
       <c r="AA34" s="63"/>
-      <c r="AB34" s="63"/>
+      <c r="AB34" s="114"/>
       <c r="AC34" s="73"/>
       <c r="AD34" s="73"/>
       <c r="AE34" s="83"/>
@@ -19354,7 +19401,7 @@
       <c r="Y35" s="63"/>
       <c r="Z35" s="63"/>
       <c r="AA35" s="63"/>
-      <c r="AB35" s="63"/>
+      <c r="AB35" s="114"/>
       <c r="AC35" s="73"/>
       <c r="AD35" s="73"/>
       <c r="AE35" s="83"/>
@@ -20283,7 +20330,7 @@
       <c r="Y36" s="63"/>
       <c r="Z36" s="63"/>
       <c r="AA36" s="63"/>
-      <c r="AB36" s="63"/>
+      <c r="AB36" s="114"/>
       <c r="AC36" s="73"/>
       <c r="AD36" s="73"/>
       <c r="AE36" s="83"/>
@@ -21212,7 +21259,7 @@
       <c r="Y37" s="63"/>
       <c r="Z37" s="63"/>
       <c r="AA37" s="63"/>
-      <c r="AB37" s="63"/>
+      <c r="AB37" s="114"/>
       <c r="AC37" s="73"/>
       <c r="AD37" s="73"/>
       <c r="AE37" s="83"/>
@@ -22141,7 +22188,7 @@
       <c r="Y38" s="63"/>
       <c r="Z38" s="63"/>
       <c r="AA38" s="63"/>
-      <c r="AB38" s="63"/>
+      <c r="AB38" s="114"/>
       <c r="AC38" s="73"/>
       <c r="AD38" s="73"/>
       <c r="AE38" s="83"/>
@@ -23070,7 +23117,7 @@
       <c r="Y39" s="63"/>
       <c r="Z39" s="63"/>
       <c r="AA39" s="63"/>
-      <c r="AB39" s="63"/>
+      <c r="AB39" s="114"/>
       <c r="AC39" s="73"/>
       <c r="AD39" s="73"/>
       <c r="AE39" s="83"/>
@@ -23999,7 +24046,7 @@
       <c r="Y40" s="63"/>
       <c r="Z40" s="63"/>
       <c r="AA40" s="63"/>
-      <c r="AB40" s="63"/>
+      <c r="AB40" s="114"/>
       <c r="AC40" s="73"/>
       <c r="AD40" s="73"/>
       <c r="AE40" s="83"/>
@@ -24928,7 +24975,7 @@
       <c r="Y41" s="63"/>
       <c r="Z41" s="63"/>
       <c r="AA41" s="63"/>
-      <c r="AB41" s="63"/>
+      <c r="AB41" s="114"/>
       <c r="AC41" s="73"/>
       <c r="AD41" s="73"/>
       <c r="AE41" s="83"/>
@@ -25857,7 +25904,7 @@
       <c r="Y42" s="63"/>
       <c r="Z42" s="63"/>
       <c r="AA42" s="63"/>
-      <c r="AB42" s="63"/>
+      <c r="AB42" s="114"/>
       <c r="AC42" s="73"/>
       <c r="AD42" s="73"/>
       <c r="AE42" s="83"/>
@@ -26786,7 +26833,7 @@
       <c r="Y43" s="63"/>
       <c r="Z43" s="63"/>
       <c r="AA43" s="63"/>
-      <c r="AB43" s="63"/>
+      <c r="AB43" s="114"/>
       <c r="AC43" s="73"/>
       <c r="AD43" s="73"/>
       <c r="AE43" s="83"/>
@@ -26823,7 +26870,7 @@
       <c r="Y44" s="63"/>
       <c r="Z44" s="63"/>
       <c r="AA44" s="63"/>
-      <c r="AB44" s="63"/>
+      <c r="AB44" s="114"/>
       <c r="AC44" s="73"/>
       <c r="AD44" s="73"/>
       <c r="AE44" s="83"/>
@@ -27752,7 +27799,7 @@
       <c r="Y45" s="63"/>
       <c r="Z45" s="63"/>
       <c r="AA45" s="63"/>
-      <c r="AB45" s="63"/>
+      <c r="AB45" s="114"/>
       <c r="AC45" s="73"/>
       <c r="AD45" s="73"/>
       <c r="AE45" s="83"/>
@@ -28682,7 +28729,7 @@
       <c r="Y46" s="63"/>
       <c r="Z46" s="63"/>
       <c r="AA46" s="63"/>
-      <c r="AB46" s="63"/>
+      <c r="AB46" s="114"/>
       <c r="AC46" s="73"/>
       <c r="AD46" s="73"/>
       <c r="AE46" s="83"/>
@@ -29611,7 +29658,7 @@
       <c r="Y47" s="63"/>
       <c r="Z47" s="63"/>
       <c r="AA47" s="63"/>
-      <c r="AB47" s="63"/>
+      <c r="AB47" s="114"/>
       <c r="AC47" s="73"/>
       <c r="AD47" s="73"/>
       <c r="AE47" s="83"/>
@@ -29648,7 +29695,7 @@
       <c r="Y48" s="63"/>
       <c r="Z48" s="63"/>
       <c r="AA48" s="63"/>
-      <c r="AB48" s="63"/>
+      <c r="AB48" s="114"/>
       <c r="AC48" s="73"/>
       <c r="AD48" s="73"/>
       <c r="AE48" s="83"/>
@@ -29685,7 +29732,7 @@
       <c r="Y49" s="63"/>
       <c r="Z49" s="63"/>
       <c r="AA49" s="63"/>
-      <c r="AB49" s="63"/>
+      <c r="AB49" s="114"/>
       <c r="AC49" s="73"/>
       <c r="AD49" s="73"/>
       <c r="AE49" s="83"/>
@@ -30614,7 +30661,7 @@
       <c r="Y50" s="63"/>
       <c r="Z50" s="63"/>
       <c r="AA50" s="63"/>
-      <c r="AB50" s="63"/>
+      <c r="AB50" s="114"/>
       <c r="AC50" s="73"/>
       <c r="AD50" s="73"/>
       <c r="AE50" s="83"/>
@@ -31543,7 +31590,7 @@
       <c r="Y51" s="64"/>
       <c r="Z51" s="64"/>
       <c r="AA51" s="64"/>
-      <c r="AB51" s="64"/>
+      <c r="AB51" s="115"/>
       <c r="AC51" s="74"/>
       <c r="AD51" s="74"/>
       <c r="AE51" s="84"/>
@@ -31580,7 +31627,7 @@
       <c r="Y52" s="65"/>
       <c r="Z52" s="65"/>
       <c r="AA52" s="65"/>
-      <c r="AB52" s="65"/>
+      <c r="AB52" s="116"/>
       <c r="AC52" s="75"/>
       <c r="AD52" s="75"/>
       <c r="AE52" s="85"/>
@@ -31617,7 +31664,7 @@
       <c r="Y53" s="66"/>
       <c r="Z53" s="66"/>
       <c r="AA53" s="66"/>
-      <c r="AB53" s="66"/>
+      <c r="AB53" s="115"/>
       <c r="AC53" s="76"/>
       <c r="AD53" s="76"/>
       <c r="AE53" s="86"/>
@@ -31654,7 +31701,7 @@
       <c r="Y54" s="66"/>
       <c r="Z54" s="66"/>
       <c r="AA54" s="66"/>
-      <c r="AB54" s="66"/>
+      <c r="AB54" s="115"/>
       <c r="AC54" s="76"/>
       <c r="AD54" s="76"/>
       <c r="AE54" s="86"/>
@@ -32583,7 +32630,7 @@
       <c r="Y55" s="67"/>
       <c r="Z55" s="67"/>
       <c r="AA55" s="67"/>
-      <c r="AB55" s="67"/>
+      <c r="AB55" s="115"/>
       <c r="AC55" s="77"/>
       <c r="AD55" s="77"/>
       <c r="AE55" s="87"/>
@@ -33512,7 +33559,7 @@
       <c r="Y56" s="66"/>
       <c r="Z56" s="66"/>
       <c r="AA56" s="66"/>
-      <c r="AB56" s="66"/>
+      <c r="AB56" s="115"/>
       <c r="AC56" s="76"/>
       <c r="AD56" s="76"/>
       <c r="AE56" s="86"/>
@@ -34441,7 +34488,7 @@
       <c r="Y57" s="67"/>
       <c r="Z57" s="67"/>
       <c r="AA57" s="67"/>
-      <c r="AB57" s="67"/>
+      <c r="AB57" s="115"/>
       <c r="AC57" s="77"/>
       <c r="AD57" s="77"/>
       <c r="AE57" s="87"/>
@@ -34478,7 +34525,7 @@
       <c r="Y58" s="66"/>
       <c r="Z58" s="66"/>
       <c r="AA58" s="66"/>
-      <c r="AB58" s="66"/>
+      <c r="AB58" s="115"/>
       <c r="AC58" s="76"/>
       <c r="AD58" s="76"/>
       <c r="AE58" s="86"/>
@@ -34515,7 +34562,7 @@
       <c r="Y59" s="66"/>
       <c r="Z59" s="66"/>
       <c r="AA59" s="66"/>
-      <c r="AB59" s="66"/>
+      <c r="AB59" s="115"/>
       <c r="AC59" s="76"/>
       <c r="AD59" s="76"/>
       <c r="AE59" s="86"/>
@@ -34552,7 +34599,7 @@
       <c r="Y60" s="66"/>
       <c r="Z60" s="66"/>
       <c r="AA60" s="66"/>
-      <c r="AB60" s="66"/>
+      <c r="AB60" s="115"/>
       <c r="AC60" s="76"/>
       <c r="AD60" s="76"/>
       <c r="AE60" s="86"/>
@@ -35481,7 +35528,7 @@
       <c r="Y61" s="68"/>
       <c r="Z61" s="68"/>
       <c r="AA61" s="68"/>
-      <c r="AB61" s="68"/>
+      <c r="AB61" s="115"/>
       <c r="AC61" s="78"/>
       <c r="AD61" s="78"/>
       <c r="AE61" s="88"/>
@@ -35518,7 +35565,7 @@
       <c r="Y62" s="66"/>
       <c r="Z62" s="66"/>
       <c r="AA62" s="66"/>
-      <c r="AB62" s="66"/>
+      <c r="AB62" s="115"/>
       <c r="AC62" s="76"/>
       <c r="AD62" s="76"/>
       <c r="AE62" s="86"/>
@@ -36448,7 +36495,7 @@
       <c r="Y63" s="66"/>
       <c r="Z63" s="66"/>
       <c r="AA63" s="66"/>
-      <c r="AB63" s="66"/>
+      <c r="AB63" s="115"/>
       <c r="AC63" s="76"/>
       <c r="AD63" s="76"/>
       <c r="AE63" s="86"/>
@@ -36485,7 +36532,7 @@
       <c r="Y64" s="66"/>
       <c r="Z64" s="66"/>
       <c r="AA64" s="66"/>
-      <c r="AB64" s="66"/>
+      <c r="AB64" s="115"/>
       <c r="AC64" s="76"/>
       <c r="AD64" s="76"/>
       <c r="AE64" s="86"/>
@@ -36522,7 +36569,7 @@
       <c r="Y65" s="66"/>
       <c r="Z65" s="66"/>
       <c r="AA65" s="66"/>
-      <c r="AB65" s="66"/>
+      <c r="AB65" s="115"/>
       <c r="AC65" s="76"/>
       <c r="AD65" s="76"/>
       <c r="AE65" s="86"/>
@@ -36559,7 +36606,7 @@
       <c r="Y66" s="69"/>
       <c r="Z66" s="69"/>
       <c r="AA66" s="69"/>
-      <c r="AB66" s="69"/>
+      <c r="AB66" s="116"/>
       <c r="AC66" s="79"/>
       <c r="AD66" s="79"/>
       <c r="AE66" s="89"/>
@@ -36596,7 +36643,7 @@
       <c r="Y67" s="70"/>
       <c r="Z67" s="70"/>
       <c r="AA67" s="70"/>
-      <c r="AB67" s="70"/>
+      <c r="AB67" s="117"/>
       <c r="AC67" s="80"/>
       <c r="AD67" s="80"/>
       <c r="AE67" s="90"/>
@@ -36633,7 +36680,7 @@
       <c r="Y68" s="71"/>
       <c r="Z68" s="71"/>
       <c r="AA68" s="71"/>
-      <c r="AB68" s="71"/>
+      <c r="AB68" s="117"/>
       <c r="AC68" s="81"/>
       <c r="AD68" s="81"/>
       <c r="AE68" s="91"/>
@@ -36670,7 +36717,7 @@
       <c r="Y69" s="71"/>
       <c r="Z69" s="71"/>
       <c r="AA69" s="71"/>
-      <c r="AB69" s="71"/>
+      <c r="AB69" s="117"/>
       <c r="AC69" s="81"/>
       <c r="AD69" s="81"/>
       <c r="AE69" s="91"/>
@@ -36707,7 +36754,7 @@
       <c r="Y70" s="71"/>
       <c r="Z70" s="71"/>
       <c r="AA70" s="71"/>
-      <c r="AB70" s="71"/>
+      <c r="AB70" s="117"/>
       <c r="AC70" s="81"/>
       <c r="AD70" s="81"/>
       <c r="AE70" s="91"/>
@@ -36744,7 +36791,7 @@
       <c r="Y71" s="71"/>
       <c r="Z71" s="71"/>
       <c r="AA71" s="71"/>
-      <c r="AB71" s="71"/>
+      <c r="AB71" s="117"/>
       <c r="AC71" s="81"/>
       <c r="AD71" s="81"/>
       <c r="AE71" s="91"/>
@@ -36781,7 +36828,7 @@
       <c r="Y72" s="71"/>
       <c r="Z72" s="71"/>
       <c r="AA72" s="71"/>
-      <c r="AB72" s="71"/>
+      <c r="AB72" s="117"/>
       <c r="AC72" s="81"/>
       <c r="AD72" s="81"/>
       <c r="AE72" s="91"/>
@@ -36818,7 +36865,7 @@
       <c r="Y73" s="71"/>
       <c r="Z73" s="71"/>
       <c r="AA73" s="71"/>
-      <c r="AB73" s="71"/>
+      <c r="AB73" s="117"/>
       <c r="AC73" s="81"/>
       <c r="AD73" s="81"/>
       <c r="AE73" s="91"/>

</xml_diff>